<commit_message>
Till Before and After Hierarchy
Config Annotation without group execution
</commit_message>
<xml_diff>
--- a/src/test/resources/testScriptData.xlsx
+++ b/src/test/resources/testScriptData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hritik\git\repository\vtiger-crm-m8\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE6B828A-8D84-4DCB-BFF3-5054B52575FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68872548-D2CC-437D-9253-0008D08F142D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -183,7 +183,7 @@
     <t>Negotiation/Review</t>
   </si>
   <si>
-    <t>awp677</t>
+    <t>awp719</t>
   </si>
 </sst>
 </file>

</xml_diff>